<commit_message>
New code modification on MpesaStatements
</commit_message>
<xml_diff>
--- a/datasets/MpesaStatements.xlsx
+++ b/datasets/MpesaStatements.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/briankimanzi/Documents/programming Languages/PythonProgramming/JupyterNoteBook/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A65EA5-E7A8-1248-B758-14C3A71E201D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CF0887-FD85-D44A-AFA7-78D0673B2F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{97F29BDA-1623-4A46-AF7B-E17D05F1B03F}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16140" activeTab="1" xr2:uid="{97F29BDA-1623-4A46-AF7B-E17D05F1B03F}"/>
   </bookViews>
   <sheets>
     <sheet name="Mpesa Statement Raw Data" sheetId="2" r:id="rId1"/>
     <sheet name="Mpesa Staments cleaning" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="359">
   <si>
     <t>Receipt No</t>
   </si>
@@ -1110,6 +1110,9 @@
   </si>
   <si>
     <t>Details Function</t>
+  </si>
+  <si>
+    <t>Received Money</t>
   </si>
 </sst>
 </file>
@@ -8405,10 +8408,10 @@
         <v>45717.663402777776</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="str">
-        <f>IF(ISNUMBER(SEARCH("Customer Transfer", B2)),"Send Money", B2)</f>
+        <f>IF(ISNUMBER(SEARCH("Funds received", B2)), "Received Money", B2)</f>
         <v>Send Money</v>
       </c>
       <c r="D2" s="3">
@@ -8428,10 +8431,7 @@
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="str">
-        <f t="shared" ref="C3:C66" si="0">IF(ISNUMBER(SEARCH("Customer Transfer", B3)),"Send Money", B3)</f>
-        <v>M-Shwari Deposit</v>
-      </c>
+      <c r="C3" s="3"/>
       <c r="D3" s="3">
         <v>0</v>
       </c>
@@ -8447,12 +8447,9 @@
         <v>45717.607407407406</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Funds received from 0706***880 - sheila mercy ndusya</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C4" s="3"/>
       <c r="D4" s="5">
         <v>1100</v>
       </c>
@@ -8470,10 +8467,7 @@
       <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C5" s="3"/>
       <c r="D5" s="3">
         <v>0</v>
       </c>
@@ -8489,12 +8483,9 @@
         <v>45716.743530092594</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C6" s="3"/>
       <c r="D6" s="3">
         <v>0</v>
       </c>
@@ -8510,10 +8501,7 @@
       <c r="B7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>NAOMI NYAMBURA MBURU</v>
-      </c>
+      <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -8525,10 +8513,7 @@
       <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C8" s="3"/>
       <c r="D8" s="3">
         <v>0</v>
       </c>
@@ -8546,10 +8531,7 @@
       <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C9" s="3"/>
       <c r="D9" s="3">
         <v>0</v>
       </c>
@@ -8565,12 +8547,9 @@
         <v>45716.478159722225</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Funds received from 254723***863 - JOHN KIMANZI</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C10" s="3"/>
       <c r="D10" s="3">
         <v>50</v>
       </c>
@@ -8586,12 +8565,9 @@
         <v>45714.81490740741</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C11" s="3"/>
       <c r="D11" s="3">
         <v>0</v>
       </c>
@@ -8607,10 +8583,7 @@
       <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>EUNICE NYATHIRA KABURA</v>
-      </c>
+      <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -8622,10 +8595,7 @@
       <c r="B13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C13" s="3"/>
       <c r="D13" s="3">
         <v>0</v>
       </c>
@@ -8641,12 +8611,9 @@
         <v>45714.377222222225</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C14" s="3"/>
       <c r="D14" s="3">
         <v>0</v>
       </c>
@@ -8662,12 +8629,9 @@
         <v>45714.377222222225</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C15" s="3"/>
       <c r="D15" s="3">
         <v>0</v>
       </c>
@@ -8683,12 +8647,9 @@
         <v>45713.425393518519</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C16" s="3"/>
       <c r="D16" s="3">
         <v>0</v>
       </c>
@@ -8704,10 +8665,7 @@
       <c r="B17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>MICHAEL MUTHOKA</v>
-      </c>
+      <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -8719,10 +8677,7 @@
       <c r="B18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C18" s="3"/>
       <c r="D18" s="3">
         <v>0</v>
       </c>
@@ -8740,10 +8695,7 @@
       <c r="B19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C19" s="3"/>
       <c r="D19" s="3">
         <v>0</v>
       </c>
@@ -8761,10 +8713,7 @@
       <c r="B20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C20" s="3"/>
       <c r="D20" s="3">
         <v>0</v>
       </c>
@@ -8780,12 +8729,9 @@
         <v>45712.745185185187</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C21" s="3"/>
       <c r="D21" s="3">
         <v>0</v>
       </c>
@@ -8803,10 +8749,7 @@
       <c r="B22" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C22" s="3"/>
       <c r="D22" s="3">
         <v>0</v>
       </c>
@@ -8822,12 +8765,9 @@
         <v>45712.740358796298</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C23" s="3"/>
       <c r="D23" s="3">
         <v>0</v>
       </c>
@@ -8843,10 +8783,7 @@
       <c r="B24" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>NYAGEIKARO JOSEPHAT OSORO</v>
-      </c>
+      <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -8858,10 +8795,7 @@
       <c r="B25" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 6627669 - Atomic Enterprises</v>
-      </c>
+      <c r="C25" s="3"/>
       <c r="D25" s="3">
         <v>0</v>
       </c>
@@ -8879,10 +8813,7 @@
       <c r="B26" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C26" s="3"/>
       <c r="D26" s="3">
         <v>0</v>
       </c>
@@ -8900,10 +8831,7 @@
       <c r="B27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C27" s="3"/>
       <c r="D27" s="3">
         <v>0</v>
       </c>
@@ -8921,10 +8849,7 @@
       <c r="B28" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C28" s="3"/>
       <c r="D28" s="3">
         <v>0</v>
       </c>
@@ -8942,10 +8867,7 @@
       <c r="B29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C29" s="3"/>
       <c r="D29" s="3">
         <v>0</v>
       </c>
@@ -8963,10 +8885,7 @@
       <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 6502951 - Ronex Mogaka Ondimu</v>
-      </c>
+      <c r="C30" s="3"/>
       <c r="D30" s="3">
         <v>0</v>
       </c>
@@ -8984,10 +8903,7 @@
       <c r="B31" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C31" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C31" s="3"/>
       <c r="D31" s="3">
         <v>0</v>
       </c>
@@ -9003,12 +8919,9 @@
         <v>45711.915590277778</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Funds received from 0799***984 - bridgit kavutha mulinge</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C32" s="3"/>
       <c r="D32" s="3">
         <v>50</v>
       </c>
@@ -9026,10 +8939,7 @@
       <c r="B33" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C33" s="3"/>
       <c r="D33" s="3">
         <v>0</v>
       </c>
@@ -9047,10 +8957,7 @@
       <c r="B34" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C34" s="3"/>
       <c r="D34" s="3">
         <v>0</v>
       </c>
@@ -9068,10 +8975,7 @@
       <c r="B35" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 6502951 - Ronex Mogaka Ondimu</v>
-      </c>
+      <c r="C35" s="3"/>
       <c r="D35" s="3">
         <v>0</v>
       </c>
@@ -9089,10 +8993,7 @@
       <c r="B36" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C36" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C36" s="3"/>
       <c r="D36" s="3">
         <v>0</v>
       </c>
@@ -9108,12 +9009,9 @@
         <v>45710.507789351854</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C37" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Funds received from 254722***289 -</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C37" s="3"/>
       <c r="D37" s="5">
         <v>2000</v>
       </c>
@@ -9129,10 +9027,7 @@
       <c r="B38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>FELISTUS NGIE</v>
-      </c>
+      <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -9144,10 +9039,7 @@
       <c r="B39" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C39" s="3"/>
       <c r="D39" s="3">
         <v>0</v>
       </c>
@@ -9165,10 +9057,7 @@
       <c r="B40" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C40" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C40" s="3"/>
       <c r="D40" s="3">
         <v>0</v>
       </c>
@@ -9186,10 +9075,7 @@
       <c r="B41" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C41" s="3"/>
       <c r="D41" s="3">
         <v>0</v>
       </c>
@@ -9207,10 +9093,7 @@
       <c r="B42" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C42" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C42" s="3"/>
       <c r="D42" s="3">
         <v>0</v>
       </c>
@@ -9228,10 +9111,7 @@
       <c r="B43" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C43" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C43" s="3"/>
       <c r="D43" s="3">
         <v>0</v>
       </c>
@@ -9249,10 +9129,7 @@
       <c r="B44" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C44" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 7385649 - STAR</v>
-      </c>
+      <c r="C44" s="3"/>
       <c r="D44" s="3">
         <v>0</v>
       </c>
@@ -9268,10 +9145,7 @@
       <c r="B45" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C45" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>BUTCHERY &amp; GROCERY</v>
-      </c>
+      <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -9281,12 +9155,9 @@
         <v>45707.806828703702</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C46" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C46" s="3"/>
       <c r="D46" s="3">
         <v>0</v>
       </c>
@@ -9304,10 +9175,7 @@
       <c r="B47" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C47" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C47" s="3"/>
       <c r="D47" s="3">
         <v>0</v>
       </c>
@@ -9325,10 +9193,7 @@
       <c r="B48" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C48" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C48" s="3"/>
       <c r="D48" s="3">
         <v>0</v>
       </c>
@@ -9344,12 +9209,9 @@
         <v>45707.682291666664</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C49" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Funds received from 254723***863 - JOHN KIMANZI</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C49" s="3"/>
       <c r="D49" s="3">
         <v>300</v>
       </c>
@@ -9367,10 +9229,7 @@
       <c r="B50" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C50" s="3"/>
       <c r="D50" s="3">
         <v>0</v>
       </c>
@@ -9386,10 +9245,7 @@
       <c r="B51" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C51" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>RONO</v>
-      </c>
+      <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -9401,10 +9257,7 @@
       <c r="B52" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C52" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C52" s="3"/>
       <c r="D52" s="3">
         <v>30</v>
       </c>
@@ -9422,10 +9275,7 @@
       <c r="B53" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C53" s="3"/>
       <c r="D53" s="3">
         <v>0</v>
       </c>
@@ -9443,10 +9293,7 @@
       <c r="B54" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C54" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C54" s="3"/>
       <c r="D54" s="3">
         <v>11</v>
       </c>
@@ -9464,10 +9311,7 @@
       <c r="B55" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C55" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C55" s="3"/>
       <c r="D55" s="3">
         <v>0</v>
       </c>
@@ -9485,10 +9329,7 @@
       <c r="B56" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C56" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C56" s="3"/>
       <c r="D56" s="3">
         <v>40</v>
       </c>
@@ -9506,10 +9347,7 @@
       <c r="B57" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C57" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C57" s="3"/>
       <c r="D57" s="3">
         <v>0</v>
       </c>
@@ -9525,10 +9363,7 @@
       <c r="B58" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C58" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>METHUSELAH KIPLAGAT CHUMBA 5</v>
-      </c>
+      <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -9540,10 +9375,7 @@
       <c r="B59" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C59" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C59" s="3"/>
       <c r="D59" s="3">
         <v>25</v>
       </c>
@@ -9561,10 +9393,7 @@
       <c r="B60" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C60" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C60" s="3"/>
       <c r="D60" s="3">
         <v>0</v>
       </c>
@@ -9582,10 +9411,7 @@
       <c r="B61" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C61" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C61" s="3"/>
       <c r="D61" s="3">
         <v>50</v>
       </c>
@@ -9603,10 +9429,7 @@
       <c r="B62" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C62" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Customer Payment to Small Business to 0745***678 - Virginia Njoki Maina</v>
-      </c>
+      <c r="C62" s="3"/>
       <c r="D62" s="3">
         <v>0</v>
       </c>
@@ -9624,10 +9447,7 @@
       <c r="B63" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C63" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C63" s="3"/>
       <c r="D63" s="3">
         <v>30</v>
       </c>
@@ -9645,10 +9465,7 @@
       <c r="B64" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C64" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C64" s="3"/>
       <c r="D64" s="3">
         <v>0</v>
       </c>
@@ -9666,10 +9483,7 @@
       <c r="B65" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C65" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C65" s="3"/>
       <c r="D65" s="3">
         <v>10</v>
       </c>
@@ -9687,10 +9501,7 @@
       <c r="B66" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C66" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Merchant Payment to 547648 - Novia Solutions</v>
-      </c>
+      <c r="C66" s="3"/>
       <c r="D66" s="3">
         <v>0</v>
       </c>
@@ -9708,10 +9519,7 @@
       <c r="B67" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C67" s="3" t="str">
-        <f t="shared" ref="C67:C130" si="1">IF(ISNUMBER(SEARCH("Customer Transfer", B67)),"Send Money", B67)</f>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C67" s="3"/>
       <c r="D67" s="5">
         <v>2000</v>
       </c>
@@ -9729,10 +9537,7 @@
       <c r="B68" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C68" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C68" s="3"/>
       <c r="D68" s="3">
         <v>0</v>
       </c>
@@ -9750,10 +9555,7 @@
       <c r="B69" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C69" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C69" s="3"/>
       <c r="D69" s="3">
         <v>0</v>
       </c>
@@ -9771,10 +9573,7 @@
       <c r="B70" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C70" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C70" s="3"/>
       <c r="D70" s="3">
         <v>0</v>
       </c>
@@ -9792,10 +9591,7 @@
       <c r="B71" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C71" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 747889 - JUJA</v>
-      </c>
+      <c r="C71" s="3"/>
       <c r="D71" s="3">
         <v>0</v>
       </c>
@@ -9811,10 +9607,7 @@
       <c r="B72" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C72" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>ECOMATT SUPERMARKED LTD</v>
-      </c>
+      <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -9826,10 +9619,7 @@
       <c r="B73" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C73" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C73" s="3"/>
       <c r="D73" s="3">
         <v>0</v>
       </c>
@@ -9847,10 +9637,7 @@
       <c r="B74" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C74" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C74" s="3"/>
       <c r="D74" s="3">
         <v>200</v>
       </c>
@@ -9868,10 +9655,7 @@
       <c r="B75" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C75" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 921961 - JKUAT CHRISTIAN UNION Acc. offering</v>
-      </c>
+      <c r="C75" s="3"/>
       <c r="D75" s="3">
         <v>0</v>
       </c>
@@ -9889,10 +9673,7 @@
       <c r="B76" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C76" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C76" s="3"/>
       <c r="D76" s="3">
         <v>50</v>
       </c>
@@ -9908,12 +9689,9 @@
         <v>45704.457372685189</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C77" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C77" s="3"/>
       <c r="D77" s="3">
         <v>0</v>
       </c>
@@ -9929,10 +9707,7 @@
       <c r="B78" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C78" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>MUTHONI</v>
-      </c>
+      <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
@@ -9944,10 +9719,7 @@
       <c r="B79" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C79" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C79" s="3"/>
       <c r="D79" s="3">
         <v>50</v>
       </c>
@@ -9965,10 +9737,7 @@
       <c r="B80" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C80" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C80" s="3"/>
       <c r="D80" s="3">
         <v>0</v>
       </c>
@@ -9986,10 +9755,7 @@
       <c r="B81" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C81" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C81" s="3"/>
       <c r="D81" s="3">
         <v>50</v>
       </c>
@@ -10007,10 +9773,7 @@
       <c r="B82" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C82" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C82" s="3"/>
       <c r="D82" s="3">
         <v>0</v>
       </c>
@@ -10028,10 +9791,7 @@
       <c r="B83" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C83" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C83" s="3"/>
       <c r="D83" s="3">
         <v>0</v>
       </c>
@@ -10049,10 +9809,7 @@
       <c r="B84" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C84" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C84" s="3"/>
       <c r="D84" s="3">
         <v>0</v>
       </c>
@@ -10070,10 +9827,7 @@
       <c r="B85" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C85" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C85" s="3"/>
       <c r="D85" s="3">
         <v>100</v>
       </c>
@@ -10091,10 +9845,7 @@
       <c r="B86" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C86" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C86" s="3"/>
       <c r="D86" s="3">
         <v>0</v>
       </c>
@@ -10112,10 +9863,7 @@
       <c r="B87" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C87" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C87" s="3"/>
       <c r="D87" s="3">
         <v>0</v>
       </c>
@@ -10133,10 +9881,7 @@
       <c r="B88" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C88" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 909090 - KACH  AIRTIME VENTURES Acc. 254104***496</v>
-      </c>
+      <c r="C88" s="3"/>
       <c r="D88" s="3">
         <v>0</v>
       </c>
@@ -10154,10 +9899,7 @@
       <c r="B89" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C89" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C89" s="3"/>
       <c r="D89" s="3">
         <v>50</v>
       </c>
@@ -10175,10 +9917,7 @@
       <c r="B90" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C90" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C90" s="3"/>
       <c r="D90" s="3">
         <v>0</v>
       </c>
@@ -10196,10 +9935,7 @@
       <c r="B91" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C91" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 909090 - KACH  AIRTIME VENTURES Acc. 254104***496</v>
-      </c>
+      <c r="C91" s="3"/>
       <c r="D91" s="3">
         <v>0</v>
       </c>
@@ -10215,12 +9951,9 @@
         <v>45701.948425925926</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C92" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C92" s="3"/>
       <c r="D92" s="3">
         <v>0</v>
       </c>
@@ -10236,10 +9969,7 @@
       <c r="B93" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C93" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>JAMES MUNGAI WACHIRA</v>
-      </c>
+      <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
@@ -10251,10 +9981,7 @@
       <c r="B94" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C94" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Customer Payment to Small Business to 0745***406 - OMAMBIA BENARD OBIERO</v>
-      </c>
+      <c r="C94" s="3"/>
       <c r="D94" s="3">
         <v>0</v>
       </c>
@@ -10272,10 +9999,7 @@
       <c r="B95" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C95" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C95" s="3"/>
       <c r="D95" s="3">
         <v>200</v>
       </c>
@@ -10293,10 +10017,7 @@
       <c r="B96" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C96" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 6033767 - HOSEA</v>
-      </c>
+      <c r="C96" s="3"/>
       <c r="D96" s="3">
         <v>0</v>
       </c>
@@ -10312,10 +10033,7 @@
       <c r="B97" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C97" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>KAHURA WAICHARI</v>
-      </c>
+      <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
@@ -10327,10 +10045,7 @@
       <c r="B98" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C98" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C98" s="3"/>
       <c r="D98" s="3">
         <v>20</v>
       </c>
@@ -10348,10 +10063,7 @@
       <c r="B99" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C99" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Customer Payment to Small Business to 0115***910 - Robert Mutua Wambua</v>
-      </c>
+      <c r="C99" s="3"/>
       <c r="D99" s="3">
         <v>0</v>
       </c>
@@ -10367,12 +10079,9 @@
         <v>45701.75681712963</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C100" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C100" s="3"/>
       <c r="D100" s="3">
         <v>0</v>
       </c>
@@ -10390,10 +10099,7 @@
       <c r="B101" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C101" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C101" s="3"/>
       <c r="D101" s="3">
         <v>200</v>
       </c>
@@ -10409,12 +10115,9 @@
         <v>45701.453553240739</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C102" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C102" s="3"/>
       <c r="D102" s="3">
         <v>0</v>
       </c>
@@ -10432,10 +10135,7 @@
       <c r="B103" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C103" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C103" s="3"/>
       <c r="D103" s="3">
         <v>0</v>
       </c>
@@ -10453,10 +10153,7 @@
       <c r="B104" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C104" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C104" s="3"/>
       <c r="D104" s="3">
         <v>200</v>
       </c>
@@ -10474,10 +10171,7 @@
       <c r="B105" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C105" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C105" s="3"/>
       <c r="D105" s="3">
         <v>0</v>
       </c>
@@ -10495,10 +10189,7 @@
       <c r="B106" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C106" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C106" s="3"/>
       <c r="D106" s="3">
         <v>30</v>
       </c>
@@ -10516,10 +10207,7 @@
       <c r="B107" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C107" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C107" s="3"/>
       <c r="D107" s="3">
         <v>190</v>
       </c>
@@ -10537,10 +10225,7 @@
       <c r="B108" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C108" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C108" s="3"/>
       <c r="D108" s="3">
         <v>0</v>
       </c>
@@ -10558,10 +10243,7 @@
       <c r="B109" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C109" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 7507293 - STELLAH</v>
-      </c>
+      <c r="C109" s="3"/>
       <c r="D109" s="3">
         <v>0</v>
       </c>
@@ -10577,10 +10259,7 @@
       <c r="B110" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C110" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>KEMUNTO ONGERI</v>
-      </c>
+      <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
       <c r="F110" s="3"/>
@@ -10592,10 +10271,7 @@
       <c r="B111" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C111" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C111" s="3"/>
       <c r="D111" s="3">
         <v>0</v>
       </c>
@@ -10611,12 +10287,9 @@
         <v>45700.869525462964</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C112" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C112" s="3"/>
       <c r="D112" s="3">
         <v>0</v>
       </c>
@@ -10634,10 +10307,7 @@
       <c r="B113" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="C113" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Customer Payment to Small Business to 0791***697 - Erick Githua Gicheche</v>
-      </c>
+      <c r="C113" s="3"/>
       <c r="D113" s="3">
         <v>0</v>
       </c>
@@ -10655,10 +10325,7 @@
       <c r="B114" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C114" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C114" s="3"/>
       <c r="D114" s="3">
         <v>200</v>
       </c>
@@ -10676,10 +10343,7 @@
       <c r="B115" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C115" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 247247 - Equity Paybill Account Acc. 0722***141</v>
-      </c>
+      <c r="C115" s="3"/>
       <c r="D115" s="3">
         <v>0</v>
       </c>
@@ -10695,12 +10359,9 @@
         <v>45700.861481481479</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C116" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C116" s="3"/>
       <c r="D116" s="3">
         <v>0</v>
       </c>
@@ -10716,12 +10377,9 @@
         <v>45700.861481481479</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C117" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C117" s="3"/>
       <c r="D117" s="3">
         <v>0</v>
       </c>
@@ -10737,10 +10395,7 @@
       <c r="B118" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C118" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>BERYL AUMA</v>
-      </c>
+      <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
       <c r="F118" s="3"/>
@@ -10752,10 +10407,7 @@
       <c r="B119" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C119" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C119" s="3"/>
       <c r="D119" s="3">
         <v>500</v>
       </c>
@@ -10773,10 +10425,7 @@
       <c r="B120" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C120" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C120" s="3"/>
       <c r="D120" s="3">
         <v>0</v>
       </c>
@@ -10794,10 +10443,7 @@
       <c r="B121" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C121" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C121" s="3"/>
       <c r="D121" s="3">
         <v>0</v>
       </c>
@@ -10815,10 +10461,7 @@
       <c r="B122" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C122" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C122" s="3"/>
       <c r="D122" s="3">
         <v>50</v>
       </c>
@@ -10836,10 +10479,7 @@
       <c r="B123" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C123" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 6862957 - LOISE</v>
-      </c>
+      <c r="C123" s="3"/>
       <c r="D123" s="3">
         <v>0</v>
       </c>
@@ -10855,10 +10495,7 @@
       <c r="B124" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C124" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>MBUGUA 2</v>
-      </c>
+      <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
       <c r="F124" s="3"/>
@@ -10870,10 +10507,7 @@
       <c r="B125" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C125" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C125" s="3"/>
       <c r="D125" s="3">
         <v>0</v>
       </c>
@@ -10891,10 +10525,7 @@
       <c r="B126" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C126" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C126" s="3"/>
       <c r="D126" s="3">
         <v>100</v>
       </c>
@@ -10912,10 +10543,7 @@
       <c r="B127" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C127" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C127" s="3"/>
       <c r="D127" s="3">
         <v>0</v>
       </c>
@@ -10933,10 +10561,7 @@
       <c r="B128" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C128" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 596742 - RUTH NJERI MUNGAI 1</v>
-      </c>
+      <c r="C128" s="3"/>
       <c r="D128" s="3">
         <v>0</v>
       </c>
@@ -10954,10 +10579,7 @@
       <c r="B129" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C129" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C129" s="3"/>
       <c r="D129" s="3">
         <v>200</v>
       </c>
@@ -10975,10 +10597,7 @@
       <c r="B130" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C130" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Merchant Payment to 596742 - RUTH NJERI MUNGAI 1</v>
-      </c>
+      <c r="C130" s="3"/>
       <c r="D130" s="3">
         <v>0</v>
       </c>
@@ -10994,12 +10613,9 @@
         <v>45699.818078703705</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C131" s="3" t="str">
-        <f t="shared" ref="C131:C194" si="2">IF(ISNUMBER(SEARCH("Customer Transfer", B131)),"Send Money", B131)</f>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C131" s="3"/>
       <c r="D131" s="3">
         <v>0</v>
       </c>
@@ -11015,12 +10631,9 @@
         <v>45699.818078703705</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C132" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C132" s="3"/>
       <c r="D132" s="3">
         <v>0</v>
       </c>
@@ -11036,10 +10649,7 @@
       <c r="B133" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C133" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>CLARIS ONGONGO</v>
-      </c>
+      <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="3"/>
       <c r="F133" s="3"/>
@@ -11051,10 +10661,7 @@
       <c r="B134" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C134" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C134" s="3"/>
       <c r="D134" s="3">
         <v>200</v>
       </c>
@@ -11072,10 +10679,7 @@
       <c r="B135" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C135" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>M-Shwari Deposit</v>
-      </c>
+      <c r="C135" s="3"/>
       <c r="D135" s="3">
         <v>0</v>
       </c>
@@ -11093,10 +10697,7 @@
       <c r="B136" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C136" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Business Payment from 547701 - National Bank Bulk Payment via API. Original conversation ID is NBKM50420255458.</v>
-      </c>
+      <c r="C136" s="3"/>
       <c r="D136" s="5">
         <v>4850</v>
       </c>
@@ -11114,10 +10715,7 @@
       <c r="B137" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C137" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C137" s="3"/>
       <c r="D137" s="3">
         <v>0</v>
       </c>
@@ -11133,12 +10731,9 @@
         <v>45698.675694444442</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C138" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C138" s="3"/>
       <c r="D138" s="3">
         <v>0</v>
       </c>
@@ -11156,10 +10751,7 @@
       <c r="B139" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C139" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C139" s="3"/>
       <c r="D139" s="3">
         <v>0</v>
       </c>
@@ -11175,12 +10767,9 @@
         <v>45698.66238425926</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C140" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Funds received from 254718***450 Gideon Kipamet Kaiyian</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C140" s="3"/>
       <c r="D140" s="3">
         <v>50</v>
       </c>
@@ -11198,10 +10787,7 @@
       <c r="B141" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="C141" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Customer Payment to Small Business to 0794***587 - HENRY NJUGUNA WAMBUI</v>
-      </c>
+      <c r="C141" s="3"/>
       <c r="D141" s="3">
         <v>0</v>
       </c>
@@ -11219,10 +10805,7 @@
       <c r="B142" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C142" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C142" s="3"/>
       <c r="D142" s="3">
         <v>0</v>
       </c>
@@ -11240,10 +10823,7 @@
       <c r="B143" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C143" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C143" s="3"/>
       <c r="D143" s="3">
         <v>0</v>
       </c>
@@ -11261,10 +10841,7 @@
       <c r="B144" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C144" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C144" s="3"/>
       <c r="D144" s="3">
         <v>0</v>
       </c>
@@ -11282,10 +10859,7 @@
       <c r="B145" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C145" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C145" s="3"/>
       <c r="D145" s="3">
         <v>0</v>
       </c>
@@ -11303,10 +10877,7 @@
       <c r="B146" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C146" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C146" s="3"/>
       <c r="D146" s="3">
         <v>0</v>
       </c>
@@ -11322,12 +10893,9 @@
         <v>45697.848495370374</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C147" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C147" s="3"/>
       <c r="D147" s="3">
         <v>0</v>
       </c>
@@ -11343,12 +10911,9 @@
         <v>45697.848495370374</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="C148" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C148" s="3"/>
       <c r="D148" s="3">
         <v>0</v>
       </c>
@@ -11366,10 +10931,7 @@
       <c r="B149" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C149" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C149" s="3"/>
       <c r="D149" s="3">
         <v>0</v>
       </c>
@@ -11385,12 +10947,9 @@
         <v>45697.510694444441</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C150" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Funds received from 254722***289 -</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C150" s="3"/>
       <c r="D150" s="3">
         <v>300</v>
       </c>
@@ -11408,10 +10967,7 @@
       <c r="B151" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C151" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C151" s="3"/>
       <c r="D151" s="3">
         <v>0</v>
       </c>
@@ -11429,10 +10985,7 @@
       <c r="B152" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C152" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C152" s="3"/>
       <c r="D152" s="3">
         <v>0</v>
       </c>
@@ -11450,10 +11003,7 @@
       <c r="B153" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C153" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C153" s="3"/>
       <c r="D153" s="3">
         <v>0</v>
       </c>
@@ -11471,10 +11021,7 @@
       <c r="B154" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C154" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C154" s="3"/>
       <c r="D154" s="3">
         <v>0</v>
       </c>
@@ -11492,10 +11039,7 @@
       <c r="B155" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C155" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C155" s="3"/>
       <c r="D155" s="3">
         <v>0</v>
       </c>
@@ -11513,10 +11057,7 @@
       <c r="B156" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C156" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C156" s="3"/>
       <c r="D156" s="3">
         <v>0</v>
       </c>
@@ -11534,10 +11075,7 @@
       <c r="B157" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C157" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C157" s="3"/>
       <c r="D157" s="3">
         <v>0</v>
       </c>
@@ -11555,10 +11093,7 @@
       <c r="B158" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C158" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C158" s="3"/>
       <c r="D158" s="3">
         <v>0</v>
       </c>
@@ -11576,10 +11111,7 @@
       <c r="B159" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C159" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C159" s="3"/>
       <c r="D159" s="3">
         <v>0</v>
       </c>
@@ -11597,10 +11129,7 @@
       <c r="B160" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C160" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C160" s="3"/>
       <c r="D160" s="3">
         <v>0</v>
       </c>
@@ -11616,12 +11145,9 @@
         <v>45695.720925925925</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C161" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C161" s="3"/>
       <c r="D161" s="3">
         <v>0</v>
       </c>
@@ -11639,10 +11165,7 @@
       <c r="B162" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C162" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C162" s="3"/>
       <c r="D162" s="3">
         <v>0</v>
       </c>
@@ -11660,10 +11183,7 @@
       <c r="B163" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C163" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C163" s="3"/>
       <c r="D163" s="3">
         <v>0</v>
       </c>
@@ -11681,10 +11201,7 @@
       <c r="B164" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C164" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C164" s="3"/>
       <c r="D164" s="3">
         <v>0</v>
       </c>
@@ -11702,10 +11219,7 @@
       <c r="B165" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C165" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C165" s="3"/>
       <c r="D165" s="3">
         <v>0</v>
       </c>
@@ -11721,12 +11235,9 @@
         <v>45693.82366898148</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C166" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C166" s="3"/>
       <c r="D166" s="3">
         <v>0</v>
       </c>
@@ -11742,12 +11253,9 @@
         <v>45693.821377314816</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C167" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C167" s="3"/>
       <c r="D167" s="3">
         <v>0</v>
       </c>
@@ -11765,10 +11273,7 @@
       <c r="B168" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C168" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Customer Payment to Small Business to</v>
-      </c>
+      <c r="C168" s="3"/>
       <c r="D168" s="3">
         <v>0</v>
       </c>
@@ -11784,10 +11289,7 @@
       <c r="B169" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C169" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>254722***209 - KELLEN NYAMBURA</v>
-      </c>
+      <c r="C169" s="3"/>
       <c r="D169" s="3"/>
       <c r="E169" s="3"/>
       <c r="F169" s="3"/>
@@ -11797,10 +11299,7 @@
       <c r="B170" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C170" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>MWANGI</v>
-      </c>
+      <c r="C170" s="3"/>
       <c r="D170" s="3"/>
       <c r="E170" s="3"/>
       <c r="F170" s="3"/>
@@ -11812,10 +11311,7 @@
       <c r="B171" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C171" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C171" s="3"/>
       <c r="D171" s="3">
         <v>0</v>
       </c>
@@ -11833,10 +11329,7 @@
       <c r="B172" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C172" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C172" s="3"/>
       <c r="D172" s="3">
         <v>0</v>
       </c>
@@ -11854,10 +11347,7 @@
       <c r="B173" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C173" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C173" s="3"/>
       <c r="D173" s="3">
         <v>0</v>
       </c>
@@ -11875,10 +11365,7 @@
       <c r="B174" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C174" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C174" s="3"/>
       <c r="D174" s="3">
         <v>0</v>
       </c>
@@ -11894,12 +11381,9 @@
         <v>45692.386990740742</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C175" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C175" s="3"/>
       <c r="D175" s="3">
         <v>0</v>
       </c>
@@ -11917,10 +11401,7 @@
       <c r="B176" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C176" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C176" s="3"/>
       <c r="D176" s="3">
         <v>0</v>
       </c>
@@ -11936,12 +11417,9 @@
         <v>45691.843993055554</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C177" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C177" s="3"/>
       <c r="D177" s="3">
         <v>0</v>
       </c>
@@ -11959,10 +11437,7 @@
       <c r="B178" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C178" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C178" s="3"/>
       <c r="D178" s="3">
         <v>0</v>
       </c>
@@ -11980,10 +11455,7 @@
       <c r="B179" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C179" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 6502951 - Ronex Mogaka Ondimu</v>
-      </c>
+      <c r="C179" s="3"/>
       <c r="D179" s="3">
         <v>0</v>
       </c>
@@ -12001,10 +11473,7 @@
       <c r="B180" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C180" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C180" s="3"/>
       <c r="D180" s="3">
         <v>0</v>
       </c>
@@ -12022,10 +11491,7 @@
       <c r="B181" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C181" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C181" s="3"/>
       <c r="D181" s="3">
         <v>0</v>
       </c>
@@ -12043,10 +11509,7 @@
       <c r="B182" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C182" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C182" s="3"/>
       <c r="D182" s="3">
         <v>0</v>
       </c>
@@ -12064,10 +11527,7 @@
       <c r="B183" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C183" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C183" s="3"/>
       <c r="D183" s="3">
         <v>0</v>
       </c>
@@ -12085,10 +11545,7 @@
       <c r="B184" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C184" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C184" s="3"/>
       <c r="D184" s="3">
         <v>0</v>
       </c>
@@ -12106,10 +11563,7 @@
       <c r="B185" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C185" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C185" s="3"/>
       <c r="D185" s="3">
         <v>0</v>
       </c>
@@ -12127,10 +11581,7 @@
       <c r="B186" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C186" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C186" s="3"/>
       <c r="D186" s="3">
         <v>0</v>
       </c>
@@ -12148,10 +11599,7 @@
       <c r="B187" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C187" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 6502951 - Ronex Mogaka Ondimu</v>
-      </c>
+      <c r="C187" s="3"/>
       <c r="D187" s="3">
         <v>0</v>
       </c>
@@ -12169,10 +11617,7 @@
       <c r="B188" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C188" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C188" s="3"/>
       <c r="D188" s="3">
         <v>0</v>
       </c>
@@ -12188,12 +11633,9 @@
         <v>45689.316168981481</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C189" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Funds received from 254722***289 -</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C189" s="3"/>
       <c r="D189" s="5">
         <v>1500</v>
       </c>
@@ -12211,10 +11653,7 @@
       <c r="B190" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C190" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C190" s="3"/>
       <c r="D190" s="3">
         <v>0</v>
       </c>
@@ -12232,10 +11671,7 @@
       <c r="B191" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C191" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C191" s="3"/>
       <c r="D191" s="3">
         <v>0</v>
       </c>
@@ -12253,10 +11689,7 @@
       <c r="B192" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C192" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C192" s="3"/>
       <c r="D192" s="3">
         <v>0</v>
       </c>
@@ -12272,12 +11705,9 @@
         <v>45686.707754629628</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C193" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C193" s="3"/>
       <c r="D193" s="3">
         <v>0</v>
       </c>
@@ -12295,10 +11725,7 @@
       <c r="B194" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C194" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C194" s="3"/>
       <c r="D194" s="3">
         <v>0</v>
       </c>
@@ -12316,10 +11743,7 @@
       <c r="B195" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C195" s="3" t="str">
-        <f t="shared" ref="C195:C258" si="3">IF(ISNUMBER(SEARCH("Customer Transfer", B195)),"Send Money", B195)</f>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C195" s="3"/>
       <c r="D195" s="3">
         <v>0</v>
       </c>
@@ -12337,10 +11761,7 @@
       <c r="B196" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C196" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C196" s="3"/>
       <c r="D196" s="3">
         <v>0</v>
       </c>
@@ -12358,10 +11779,7 @@
       <c r="B197" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C197" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C197" s="3"/>
       <c r="D197" s="3">
         <v>0</v>
       </c>
@@ -12379,10 +11797,7 @@
       <c r="B198" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C198" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C198" s="3"/>
       <c r="D198" s="3">
         <v>0</v>
       </c>
@@ -12400,10 +11815,7 @@
       <c r="B199" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C199" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C199" s="3"/>
       <c r="D199" s="3">
         <v>0</v>
       </c>
@@ -12419,12 +11831,9 @@
         <v>45684.794687499998</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C200" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C200" s="3"/>
       <c r="D200" s="3">
         <v>0</v>
       </c>
@@ -12442,10 +11851,7 @@
       <c r="B201" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C201" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C201" s="3"/>
       <c r="D201" s="3">
         <v>0</v>
       </c>
@@ -12463,10 +11869,7 @@
       <c r="B202" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C202" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C202" s="3"/>
       <c r="D202" s="3">
         <v>0</v>
       </c>
@@ -12482,12 +11885,9 @@
         <v>45684.778287037036</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C203" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Funds received from 254723***863 - JOHN KIMANZI</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C203" s="3"/>
       <c r="D203" s="3">
         <v>400</v>
       </c>
@@ -12505,10 +11905,7 @@
       <c r="B204" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C204" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C204" s="3"/>
       <c r="D204" s="3">
         <v>0</v>
       </c>
@@ -12524,12 +11921,9 @@
         <v>45682.745763888888</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C205" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C205" s="3"/>
       <c r="D205" s="3">
         <v>0</v>
       </c>
@@ -12547,10 +11941,7 @@
       <c r="B206" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C206" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C206" s="3"/>
       <c r="D206" s="3">
         <v>0</v>
       </c>
@@ -12568,10 +11959,7 @@
       <c r="B207" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C207" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C207" s="3"/>
       <c r="D207" s="3">
         <v>0</v>
       </c>
@@ -12589,10 +11977,7 @@
       <c r="B208" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C208" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C208" s="3"/>
       <c r="D208" s="3">
         <v>0</v>
       </c>
@@ -12610,10 +11995,7 @@
       <c r="B209" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C209" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C209" s="3"/>
       <c r="D209" s="3">
         <v>0</v>
       </c>
@@ -12631,10 +12013,7 @@
       <c r="B210" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="C210" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill to 522533 - Lipa na KCB Acc. 6060082</v>
-      </c>
+      <c r="C210" s="3"/>
       <c r="D210" s="3">
         <v>0</v>
       </c>
@@ -12650,12 +12029,9 @@
         <v>45681.433078703703</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="C211" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C211" s="3"/>
       <c r="D211" s="3">
         <v>0</v>
       </c>
@@ -12673,10 +12049,7 @@
       <c r="B212" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C212" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C212" s="3"/>
       <c r="D212" s="3">
         <v>0</v>
       </c>
@@ -12694,10 +12067,7 @@
       <c r="B213" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C213" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C213" s="3"/>
       <c r="D213" s="3">
         <v>0</v>
       </c>
@@ -12715,10 +12085,7 @@
       <c r="B214" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C214" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C214" s="3"/>
       <c r="D214" s="3">
         <v>0</v>
       </c>
@@ -12736,10 +12103,7 @@
       <c r="B215" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C215" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C215" s="3"/>
       <c r="D215" s="3">
         <v>0</v>
       </c>
@@ -12757,10 +12121,7 @@
       <c r="B216" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C216" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C216" s="3"/>
       <c r="D216" s="3">
         <v>0</v>
       </c>
@@ -12778,10 +12139,7 @@
       <c r="B217" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C217" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C217" s="3"/>
       <c r="D217" s="3">
         <v>0</v>
       </c>
@@ -12799,10 +12157,7 @@
       <c r="B218" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C218" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C218" s="3"/>
       <c r="D218" s="3">
         <v>0</v>
       </c>
@@ -12820,10 +12175,7 @@
       <c r="B219" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C219" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 6627669 - Atomic Enterprises</v>
-      </c>
+      <c r="C219" s="3"/>
       <c r="D219" s="3">
         <v>0</v>
       </c>
@@ -12841,10 +12193,7 @@
       <c r="B220" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C220" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4076749 - TINGG Acc. 254104***496</v>
-      </c>
+      <c r="C220" s="3"/>
       <c r="D220" s="3">
         <v>0</v>
       </c>
@@ -12862,10 +12211,7 @@
       <c r="B221" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C221" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C221" s="3"/>
       <c r="D221" s="3">
         <v>0</v>
       </c>
@@ -12883,10 +12229,7 @@
       <c r="B222" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C222" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C222" s="3"/>
       <c r="D222" s="3">
         <v>0</v>
       </c>
@@ -12904,10 +12247,7 @@
       <c r="B223" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="C223" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1120883103</v>
-      </c>
+      <c r="C223" s="3"/>
       <c r="D223" s="3">
         <v>0</v>
       </c>
@@ -12925,10 +12265,7 @@
       <c r="B224" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C224" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C224" s="3"/>
       <c r="D224" s="3">
         <v>0</v>
       </c>
@@ -12946,10 +12283,7 @@
       <c r="B225" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="C225" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 667505 - FRANCIS MAINA NJIHIA.</v>
-      </c>
+      <c r="C225" s="3"/>
       <c r="D225" s="3">
         <v>0</v>
       </c>
@@ -12967,10 +12301,7 @@
       <c r="B226" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C226" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C226" s="3"/>
       <c r="D226" s="3">
         <v>0</v>
       </c>
@@ -12988,10 +12319,7 @@
       <c r="B227" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C227" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill to 909090 - KACH  AIRTIME VENTURES Acc. 254104***496</v>
-      </c>
+      <c r="C227" s="3"/>
       <c r="D227" s="3">
         <v>0</v>
       </c>
@@ -13009,10 +12337,7 @@
       <c r="B228" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C228" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C228" s="3"/>
       <c r="D228" s="3">
         <v>0</v>
       </c>
@@ -13030,10 +12355,7 @@
       <c r="B229" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C229" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1120110105</v>
-      </c>
+      <c r="C229" s="3"/>
       <c r="D229" s="3">
         <v>0</v>
       </c>
@@ -13051,10 +12373,7 @@
       <c r="B230" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C230" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C230" s="3"/>
       <c r="D230" s="3">
         <v>0</v>
       </c>
@@ -13072,10 +12391,7 @@
       <c r="B231" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C231" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C231" s="3"/>
       <c r="D231" s="3">
         <v>0</v>
       </c>
@@ -13093,10 +12409,7 @@
       <c r="B232" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C232" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Deposit of Funds at Agent Till 332527 -</v>
-      </c>
+      <c r="C232" s="3"/>
       <c r="D232" s="5">
         <v>1000</v>
       </c>
@@ -13112,10 +12425,7 @@
       <c r="B233" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="C233" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Kool phones STEVE SHOP JOYLAND MRT JUJA</v>
-      </c>
+      <c r="C233" s="3"/>
       <c r="D233" s="3"/>
       <c r="E233" s="3"/>
       <c r="F233" s="3"/>
@@ -13125,12 +12435,9 @@
         <v>45675.491076388891</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C234" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Funds received from 254722***289 -</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="C234" s="3"/>
       <c r="D234" s="5">
         <v>1500</v>
       </c>
@@ -13148,10 +12455,7 @@
       <c r="B235" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C235" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C235" s="3"/>
       <c r="D235" s="3">
         <v>0</v>
       </c>
@@ -13169,10 +12473,7 @@
       <c r="B236" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C236" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C236" s="3"/>
       <c r="D236" s="3">
         <v>0</v>
       </c>
@@ -13190,10 +12491,7 @@
       <c r="B237" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C237" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C237" s="3"/>
       <c r="D237" s="3">
         <v>41</v>
       </c>
@@ -13211,10 +12509,7 @@
       <c r="B238" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C238" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C238" s="3"/>
       <c r="D238" s="3">
         <v>0</v>
       </c>
@@ -13232,10 +12527,7 @@
       <c r="B239" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C239" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C239" s="3"/>
       <c r="D239" s="3">
         <v>100</v>
       </c>
@@ -13251,12 +12543,9 @@
         <v>45674.469837962963</v>
       </c>
       <c r="B240" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C240" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C240" s="3"/>
       <c r="D240" s="3">
         <v>0</v>
       </c>
@@ -13272,12 +12561,9 @@
         <v>45674.469837962963</v>
       </c>
       <c r="B241" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="C241" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C241" s="3"/>
       <c r="D241" s="3">
         <v>0</v>
       </c>
@@ -13293,10 +12579,7 @@
       <c r="B242" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="C242" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>FAITH WANGARI NJOROGE</v>
-      </c>
+      <c r="C242" s="3"/>
       <c r="D242" s="3"/>
       <c r="E242" s="3"/>
       <c r="F242" s="3"/>
@@ -13308,10 +12591,7 @@
       <c r="B243" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C243" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C243" s="3"/>
       <c r="D243" s="3">
         <v>7</v>
       </c>
@@ -13329,10 +12609,7 @@
       <c r="B244" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C244" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C244" s="3"/>
       <c r="D244" s="3">
         <v>170</v>
       </c>
@@ -13350,10 +12627,7 @@
       <c r="B245" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="C245" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Customer Payment to Small Business to 0112***535 - Alex Onduko Mogaka</v>
-      </c>
+      <c r="C245" s="3"/>
       <c r="D245" s="3">
         <v>0</v>
       </c>
@@ -13371,10 +12645,7 @@
       <c r="B246" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C246" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C246" s="3"/>
       <c r="D246" s="3">
         <v>50</v>
       </c>
@@ -13392,10 +12663,7 @@
       <c r="B247" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C247" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C247" s="3"/>
       <c r="D247" s="3">
         <v>0</v>
       </c>
@@ -13413,10 +12681,7 @@
       <c r="B248" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="C248" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1112880256</v>
-      </c>
+      <c r="C248" s="3"/>
       <c r="D248" s="3">
         <v>0</v>
       </c>
@@ -13434,10 +12699,7 @@
       <c r="B249" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C249" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C249" s="3"/>
       <c r="D249" s="3">
         <v>12</v>
       </c>
@@ -13455,10 +12717,7 @@
       <c r="B250" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C250" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C250" s="3"/>
       <c r="D250" s="3">
         <v>0</v>
       </c>
@@ -13476,10 +12735,7 @@
       <c r="B251" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C251" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1111700185</v>
-      </c>
+      <c r="C251" s="3"/>
       <c r="D251" s="3">
         <v>0</v>
       </c>
@@ -13497,10 +12753,7 @@
       <c r="B252" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C252" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 6502951 - Ronex Mogaka Ondimu</v>
-      </c>
+      <c r="C252" s="3"/>
       <c r="D252" s="3">
         <v>0</v>
       </c>
@@ -13518,10 +12771,7 @@
       <c r="B253" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C253" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C253" s="3"/>
       <c r="D253" s="3">
         <v>120</v>
       </c>
@@ -13539,10 +12789,7 @@
       <c r="B254" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C254" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 547648 - Novia Solutions</v>
-      </c>
+      <c r="C254" s="3"/>
       <c r="D254" s="3">
         <v>0</v>
       </c>
@@ -13560,10 +12807,7 @@
       <c r="B255" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C255" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C255" s="3"/>
       <c r="D255" s="5">
         <v>2500</v>
       </c>
@@ -13581,10 +12825,7 @@
       <c r="B256" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C256" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C256" s="3"/>
       <c r="D256" s="3">
         <v>0</v>
       </c>
@@ -13602,10 +12843,7 @@
       <c r="B257" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="C257" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1109346985</v>
-      </c>
+      <c r="C257" s="3"/>
       <c r="D257" s="3">
         <v>0</v>
       </c>
@@ -13623,10 +12861,7 @@
       <c r="B258" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C258" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>Merchant Payment to 7886415 -</v>
-      </c>
+      <c r="C258" s="3"/>
       <c r="D258" s="3">
         <v>0</v>
       </c>
@@ -13644,10 +12879,7 @@
       <c r="B259" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C259" s="3" t="str">
-        <f t="shared" ref="C259:C298" si="4">IF(ISNUMBER(SEARCH("Customer Transfer", B259)),"Send Money", B259)</f>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C259" s="3"/>
       <c r="D259" s="3">
         <v>0</v>
       </c>
@@ -13665,10 +12897,7 @@
       <c r="B260" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="C260" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1109335138</v>
-      </c>
+      <c r="C260" s="3"/>
       <c r="D260" s="3">
         <v>0</v>
       </c>
@@ -13686,10 +12915,7 @@
       <c r="B261" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C261" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C261" s="3"/>
       <c r="D261" s="3">
         <v>100</v>
       </c>
@@ -13707,10 +12933,7 @@
       <c r="B262" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C262" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C262" s="3"/>
       <c r="D262" s="3">
         <v>0</v>
       </c>
@@ -13728,10 +12951,7 @@
       <c r="B263" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="C263" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1108956193</v>
-      </c>
+      <c r="C263" s="3"/>
       <c r="D263" s="3">
         <v>0</v>
       </c>
@@ -13749,10 +12969,7 @@
       <c r="B264" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C264" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C264" s="3"/>
       <c r="D264" s="3">
         <v>6</v>
       </c>
@@ -13770,10 +12987,7 @@
       <c r="B265" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C265" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C265" s="3"/>
       <c r="D265" s="3">
         <v>0</v>
       </c>
@@ -13791,10 +13005,7 @@
       <c r="B266" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C266" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C266" s="3"/>
       <c r="D266" s="3">
         <v>40</v>
       </c>
@@ -13812,10 +13023,7 @@
       <c r="B267" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C267" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C267" s="3"/>
       <c r="D267" s="3">
         <v>0</v>
       </c>
@@ -13833,10 +13041,7 @@
       <c r="B268" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C268" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C268" s="3"/>
       <c r="D268" s="3">
         <v>15</v>
       </c>
@@ -13854,10 +13059,7 @@
       <c r="B269" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C269" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C269" s="3"/>
       <c r="D269" s="3">
         <v>100</v>
       </c>
@@ -13875,10 +13077,7 @@
       <c r="B270" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C270" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C270" s="3"/>
       <c r="D270" s="3">
         <v>0</v>
       </c>
@@ -13896,10 +13095,7 @@
       <c r="B271" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="C271" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1105727129</v>
-      </c>
+      <c r="C271" s="3"/>
       <c r="D271" s="3">
         <v>0</v>
       </c>
@@ -13915,12 +13111,9 @@
         <v>45671.560891203706</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C272" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C272" s="3"/>
       <c r="D272" s="3">
         <v>0</v>
       </c>
@@ -13938,10 +13131,7 @@
       <c r="B273" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C273" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C273" s="3"/>
       <c r="D273" s="3">
         <v>30</v>
       </c>
@@ -13959,10 +13149,7 @@
       <c r="B274" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C274" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C274" s="3"/>
       <c r="D274" s="3">
         <v>0</v>
       </c>
@@ -13980,10 +13167,7 @@
       <c r="B275" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="C275" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1105110448</v>
-      </c>
+      <c r="C275" s="3"/>
       <c r="D275" s="3">
         <v>0</v>
       </c>
@@ -14001,10 +13185,7 @@
       <c r="B276" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C276" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C276" s="3"/>
       <c r="D276" s="3">
         <v>22</v>
       </c>
@@ -14022,10 +13203,7 @@
       <c r="B277" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C277" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Customer Payment to Small Business to</v>
-      </c>
+      <c r="C277" s="3"/>
       <c r="D277" s="3">
         <v>0</v>
       </c>
@@ -14041,10 +13219,7 @@
       <c r="B278" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C278" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>254714***875 - EUCABETH BUYAKI</v>
-      </c>
+      <c r="C278" s="3"/>
       <c r="D278" s="3"/>
       <c r="E278" s="3"/>
       <c r="F278" s="3"/>
@@ -14054,10 +13229,7 @@
       <c r="B279" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="C279" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>KEBWARO</v>
-      </c>
+      <c r="C279" s="3"/>
       <c r="D279" s="3"/>
       <c r="E279" s="3"/>
       <c r="F279" s="3"/>
@@ -14069,10 +13241,7 @@
       <c r="B280" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C280" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C280" s="3"/>
       <c r="D280" s="3">
         <v>40</v>
       </c>
@@ -14088,12 +13257,9 @@
         <v>45670.656689814816</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C281" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C281" s="3"/>
       <c r="D281" s="3">
         <v>0</v>
       </c>
@@ -14111,10 +13277,7 @@
       <c r="B282" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C282" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C282" s="3"/>
       <c r="D282" s="3">
         <v>55</v>
       </c>
@@ -14132,10 +13295,7 @@
       <c r="B283" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C283" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Merchant Payment to 7292565 - LINUS</v>
-      </c>
+      <c r="C283" s="3"/>
       <c r="D283" s="3">
         <v>0</v>
       </c>
@@ -14153,10 +13313,7 @@
       <c r="B284" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C284" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C284" s="3"/>
       <c r="D284" s="3">
         <v>100</v>
       </c>
@@ -14174,10 +13331,7 @@
       <c r="B285" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C285" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill to 888880 - KPLC PREPAID Acc. 37165920945</v>
-      </c>
+      <c r="C285" s="3"/>
       <c r="D285" s="3">
         <v>0</v>
       </c>
@@ -14195,10 +13349,7 @@
       <c r="B286" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C286" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C286" s="3"/>
       <c r="D286" s="3">
         <v>100</v>
       </c>
@@ -14216,10 +13367,7 @@
       <c r="B287" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C287" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C287" s="3"/>
       <c r="D287" s="3">
         <v>0</v>
       </c>
@@ -14237,10 +13385,7 @@
       <c r="B288" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="C288" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1101362244</v>
-      </c>
+      <c r="C288" s="3"/>
       <c r="D288" s="3">
         <v>0</v>
       </c>
@@ -14258,10 +13403,7 @@
       <c r="B289" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C289" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C289" s="3"/>
       <c r="D289" s="3">
         <v>12</v>
       </c>
@@ -14279,10 +13421,7 @@
       <c r="B290" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C290" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Customer Payment to Small Business to 254714***909 - BETH WANGARI MWAI</v>
-      </c>
+      <c r="C290" s="3"/>
       <c r="D290" s="3">
         <v>0</v>
       </c>
@@ -14300,10 +13439,7 @@
       <c r="B291" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C291" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C291" s="3"/>
       <c r="D291" s="3">
         <v>70</v>
       </c>
@@ -14319,12 +13455,9 @@
         <v>45668.858159722222</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="C292" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Send Money</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C292" s="3"/>
       <c r="D292" s="3">
         <v>0</v>
       </c>
@@ -14340,10 +13473,7 @@
       <c r="B293" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="C293" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>PERIR WANJIRU NJUGUNA</v>
-      </c>
+      <c r="C293" s="3"/>
       <c r="D293" s="3"/>
       <c r="E293" s="3"/>
       <c r="F293" s="3"/>
@@ -14355,10 +13485,7 @@
       <c r="B294" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C294" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C294" s="3"/>
       <c r="D294" s="3">
         <v>50</v>
       </c>
@@ -14376,10 +13503,7 @@
       <c r="B295" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C295" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Charge</v>
-      </c>
+      <c r="C295" s="3"/>
       <c r="D295" s="3">
         <v>0</v>
       </c>
@@ -14397,10 +13521,7 @@
       <c r="B296" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="C296" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Pay Bill Online to 4093275 - Direct Pay Limited 1 Acc. ATL1095514765</v>
-      </c>
+      <c r="C296" s="3"/>
       <c r="D296" s="3">
         <v>0</v>
       </c>
@@ -14418,10 +13539,7 @@
       <c r="B297" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C297" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>M-Shwari Withdraw</v>
-      </c>
+      <c r="C297" s="3"/>
       <c r="D297" s="3">
         <v>50</v>
       </c>
@@ -14439,10 +13557,7 @@
       <c r="B298" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C298" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>Merchant Payment to 686190 - STEPHEN KIARIE</v>
-      </c>
+      <c r="C298" s="3"/>
       <c r="D298" s="3">
         <v>0</v>
       </c>

</xml_diff>